<commit_message>
foreclosures: Greenville 9/8 withdrawals from the current sale list + Form 4 worklist
Nine cases now withdrawn (#1, 7, 13, 15, 17, 19, 21, 22, 29); #20 deficiency
waived after approval. Seed rows carry direct docket + Journal case links;
reports/greenville-2026-09-08-form4-worklist.csv lists the 20 live cases
with blank Judgment/As-of/Per-diem columns to fill from the Form 4.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017rdAjmKGDVGAtDqQodYkcB
</commit_message>
<xml_diff>
--- a/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
+++ b/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
@@ -1649,7 +1649,11 @@
       <c r="W9" s="11" t="n"/>
       <c r="X9" s="11" t="inlineStr"/>
       <c r="Y9" s="11" t="n"/>
-      <c r="Z9" s="11" t="n"/>
+      <c r="Z9" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA9" s="11" t="n"/>
       <c r="AB9" s="11" t="n"/>
       <c r="AC9" s="9" t="inlineStr">
@@ -1743,7 +1747,11 @@
         </is>
       </c>
       <c r="Y10" s="11" t="n"/>
-      <c r="Z10" s="11" t="n"/>
+      <c r="Z10" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA10" s="11" t="n"/>
       <c r="AB10" s="14" t="inlineStr">
         <is>
@@ -1841,7 +1849,11 @@
         </is>
       </c>
       <c r="Y11" s="11" t="n"/>
-      <c r="Z11" s="11" t="n"/>
+      <c r="Z11" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA11" s="11" t="n"/>
       <c r="AB11" s="14" t="inlineStr">
         <is>
@@ -1939,7 +1951,11 @@
         </is>
       </c>
       <c r="Y12" s="11" t="n"/>
-      <c r="Z12" s="11" t="n"/>
+      <c r="Z12" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA12" s="11" t="n"/>
       <c r="AB12" s="14" t="inlineStr">
         <is>
@@ -2037,7 +2053,11 @@
         </is>
       </c>
       <c r="Y13" s="11" t="n"/>
-      <c r="Z13" s="11" t="n"/>
+      <c r="Z13" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA13" s="11" t="n"/>
       <c r="AB13" s="14" t="inlineStr">
         <is>
@@ -2117,7 +2137,11 @@
       <c r="W14" s="11" t="n"/>
       <c r="X14" s="11" t="inlineStr"/>
       <c r="Y14" s="11" t="n"/>
-      <c r="Z14" s="11" t="n"/>
+      <c r="Z14" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA14" s="11" t="n"/>
       <c r="AB14" s="11" t="n"/>
       <c r="AC14" s="9" t="inlineStr">
@@ -2193,7 +2217,11 @@
       <c r="W15" s="11" t="n"/>
       <c r="X15" s="11" t="inlineStr"/>
       <c r="Y15" s="11" t="n"/>
-      <c r="Z15" s="11" t="n"/>
+      <c r="Z15" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA15" s="11" t="n"/>
       <c r="AB15" s="11" t="n"/>
       <c r="AC15" s="9" t="inlineStr">
@@ -2287,7 +2315,11 @@
         </is>
       </c>
       <c r="Y16" s="11" t="n"/>
-      <c r="Z16" s="11" t="n"/>
+      <c r="Z16" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA16" s="11" t="n"/>
       <c r="AB16" s="14" t="inlineStr">
         <is>
@@ -2385,7 +2417,11 @@
         </is>
       </c>
       <c r="Y17" s="11" t="n"/>
-      <c r="Z17" s="11" t="n"/>
+      <c r="Z17" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA17" s="11" t="n"/>
       <c r="AB17" s="14" t="inlineStr">
         <is>
@@ -2483,7 +2519,11 @@
         </is>
       </c>
       <c r="Y18" s="11" t="n"/>
-      <c r="Z18" s="11" t="n"/>
+      <c r="Z18" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA18" s="11" t="n"/>
       <c r="AB18" s="14" t="inlineStr">
         <is>
@@ -2563,7 +2603,11 @@
       <c r="W19" s="11" t="n"/>
       <c r="X19" s="11" t="inlineStr"/>
       <c r="Y19" s="11" t="n"/>
-      <c r="Z19" s="11" t="n"/>
+      <c r="Z19" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA19" s="11" t="n"/>
       <c r="AB19" s="11" t="n"/>
       <c r="AC19" s="9" t="inlineStr">
@@ -2657,7 +2701,11 @@
         </is>
       </c>
       <c r="Y20" s="11" t="n"/>
-      <c r="Z20" s="11" t="n"/>
+      <c r="Z20" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA20" s="11" t="n"/>
       <c r="AB20" s="14" t="inlineStr">
         <is>
@@ -2689,7 +2737,7 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -2725,46 +2773,28 @@
         <v/>
       </c>
       <c r="P21" s="11" t="n"/>
-      <c r="Q21" s="12" t="n">
-        <v>363430</v>
-      </c>
+      <c r="Q21" s="12" t="n"/>
       <c r="R21" s="13">
         <f>IF(OR(Q21="",Q21=0,O21=""),"",O21/Q21)</f>
         <v/>
       </c>
-      <c r="S21" s="11" t="inlineStr">
-        <is>
-          <t>0.150</t>
-        </is>
-      </c>
-      <c r="T21" s="11" t="inlineStr">
-        <is>
-          <t>1100 (Single Family)</t>
-        </is>
-      </c>
+      <c r="S21" s="11" t="n"/>
+      <c r="T21" s="11" t="n"/>
       <c r="U21" s="11" t="n"/>
       <c r="V21" s="11" t="n"/>
-      <c r="W21" s="11" t="inlineStr">
-        <is>
-          <t>Abad Nancy</t>
-        </is>
-      </c>
-      <c r="X21" s="11" t="inlineStr">
-        <is>
-          <t>03/28/2019 $277,830</t>
-        </is>
-      </c>
+      <c r="W21" s="11" t="n"/>
+      <c r="X21" s="11" t="inlineStr"/>
       <c r="Y21" s="11" t="n"/>
-      <c r="Z21" s="11" t="n"/>
+      <c r="Z21" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA21" s="11" t="n"/>
-      <c r="AB21" s="14" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="AB21" s="11" t="n"/>
       <c r="AC21" s="9" t="inlineStr">
         <is>
-          <t>406 Sandusky Lane Simpsonville, SC 29680 — 1100 (Single Family) — 0.150 ac (Mill Pond At River Shoa). Record owner Abad Nancy. Last transfer 03/28/2019 for $277,830. County FMV $363,430.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>406 Sandusky Lane Simpsonville, SC 29680. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2883,11 @@
         </is>
       </c>
       <c r="Y22" s="11" t="n"/>
-      <c r="Z22" s="11" t="n"/>
+      <c r="Z22" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA22" s="11" t="n"/>
       <c r="AB22" s="14" t="inlineStr">
         <is>
@@ -2885,7 +2919,7 @@
       </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
@@ -2921,46 +2955,28 @@
         <v/>
       </c>
       <c r="P23" s="11" t="n"/>
-      <c r="Q23" s="12" t="n">
-        <v>555460</v>
-      </c>
+      <c r="Q23" s="12" t="n"/>
       <c r="R23" s="13">
         <f>IF(OR(Q23="",Q23=0,O23=""),"",O23/Q23)</f>
         <v/>
       </c>
-      <c r="S23" s="11" t="inlineStr">
-        <is>
-          <t>0.580</t>
-        </is>
-      </c>
-      <c r="T23" s="11" t="inlineStr">
-        <is>
-          <t>1100 (Single Family)</t>
-        </is>
-      </c>
+      <c r="S23" s="11" t="n"/>
+      <c r="T23" s="11" t="n"/>
       <c r="U23" s="11" t="n"/>
       <c r="V23" s="11" t="n"/>
-      <c r="W23" s="11" t="inlineStr">
-        <is>
-          <t>Belue Deana Ann (Jtwros)</t>
-        </is>
-      </c>
-      <c r="X23" s="11" t="inlineStr">
-        <is>
-          <t>12/26/2018 $395,710</t>
-        </is>
-      </c>
+      <c r="W23" s="11" t="n"/>
+      <c r="X23" s="11" t="inlineStr"/>
       <c r="Y23" s="11" t="n"/>
-      <c r="Z23" s="11" t="n"/>
+      <c r="Z23" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA23" s="11" t="n"/>
-      <c r="AB23" s="14" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="AB23" s="11" t="n"/>
       <c r="AC23" s="9" t="inlineStr">
         <is>
-          <t>116 Ridgewater Court Fountain Inn, SC 29644 — 1100 (Single Family) — 0.580 ac (Ridgewater). Record owner Belue Deana Ann (Jtwros). Last transfer 12/26/2018 for $395,710. County FMV $555,460.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>116 Ridgewater Court Fountain Inn, SC 29644. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3065,11 @@
         </is>
       </c>
       <c r="Y24" s="11" t="n"/>
-      <c r="Z24" s="11" t="n"/>
+      <c r="Z24" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA24" s="11" t="n"/>
       <c r="AB24" s="14" t="inlineStr">
         <is>
@@ -3129,7 +3149,11 @@
       <c r="W25" s="11" t="n"/>
       <c r="X25" s="11" t="inlineStr"/>
       <c r="Y25" s="11" t="n"/>
-      <c r="Z25" s="11" t="n"/>
+      <c r="Z25" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA25" s="11" t="n"/>
       <c r="AB25" s="11" t="n"/>
       <c r="AC25" s="9" t="inlineStr">
@@ -3223,7 +3247,11 @@
         </is>
       </c>
       <c r="Y26" s="11" t="n"/>
-      <c r="Z26" s="11" t="n"/>
+      <c r="Z26" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA26" s="11" t="n"/>
       <c r="AB26" s="14" t="inlineStr">
         <is>
@@ -3255,7 +3283,7 @@
       </c>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
@@ -3291,46 +3319,28 @@
         <v/>
       </c>
       <c r="P27" s="11" t="n"/>
-      <c r="Q27" s="12" t="n">
-        <v>173420</v>
-      </c>
+      <c r="Q27" s="12" t="n"/>
       <c r="R27" s="13">
         <f>IF(OR(Q27="",Q27=0,O27=""),"",O27/Q27)</f>
         <v/>
       </c>
-      <c r="S27" s="11" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="T27" s="11" t="inlineStr">
-        <is>
-          <t>1100 (Single Family)</t>
-        </is>
-      </c>
+      <c r="S27" s="11" t="n"/>
+      <c r="T27" s="11" t="n"/>
       <c r="U27" s="11" t="n"/>
       <c r="V27" s="11" t="n"/>
-      <c r="W27" s="11" t="inlineStr">
-        <is>
-          <t>Hammett Sylvia Merritt</t>
-        </is>
-      </c>
-      <c r="X27" s="11" t="inlineStr">
-        <is>
-          <t>06/12/2007</t>
-        </is>
-      </c>
+      <c r="W27" s="11" t="n"/>
+      <c r="X27" s="11" t="inlineStr"/>
       <c r="Y27" s="11" t="n"/>
-      <c r="Z27" s="11" t="n"/>
+      <c r="Z27" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA27" s="11" t="n"/>
-      <c r="AB27" s="14" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="AB27" s="11" t="n"/>
       <c r="AC27" s="9" t="inlineStr">
         <is>
-          <t>67 Wallace Street Greenville, SC 29605 — 1100 (Single Family) (Dunean Mills). Record owner Hammett Sylvia Merritt. Last transfer 06/12/2007. County FMV $173,420.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>67 Wallace Street Greenville, SC 29605. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -3374,7 +3384,7 @@
       </c>
       <c r="J28" s="11" t="inlineStr">
         <is>
-          <t>demanded</t>
+          <t>waived</t>
         </is>
       </c>
       <c r="K28" s="12" t="n"/>
@@ -3419,7 +3429,11 @@
         </is>
       </c>
       <c r="Y28" s="11" t="n"/>
-      <c r="Z28" s="11" t="n"/>
+      <c r="Z28" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA28" s="11" t="n"/>
       <c r="AB28" s="14" t="inlineStr">
         <is>
@@ -3428,7 +3442,7 @@
       </c>
       <c r="AC28" s="9" t="inlineStr">
         <is>
-          <t>100 N. Markley St. Greenville, SC 29601 — 6800 (Commercial Vacant ) — 0.910 ac. Record owner Greenville Hkw Llc. Last transfer 12/16/2019. County FMV $2,973,000.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>100 N. Markley St. Greenville, SC 29601 — 6800 (Commercial Vacant ) — 0.910 ac. Record owner Greenville Hkw Llc. Last transfer 12/16/2019. County FMV $2,973,000.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3499,7 +3513,11 @@
       <c r="W29" s="11" t="n"/>
       <c r="X29" s="11" t="inlineStr"/>
       <c r="Y29" s="11" t="n"/>
-      <c r="Z29" s="11" t="n"/>
+      <c r="Z29" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA29" s="11" t="n"/>
       <c r="AB29" s="11" t="n"/>
       <c r="AC29" s="9" t="inlineStr">
@@ -3575,7 +3593,11 @@
       <c r="W30" s="11" t="n"/>
       <c r="X30" s="11" t="inlineStr"/>
       <c r="Y30" s="11" t="n"/>
-      <c r="Z30" s="11" t="n"/>
+      <c r="Z30" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA30" s="11" t="n"/>
       <c r="AB30" s="11" t="n"/>
       <c r="AC30" s="9" t="inlineStr">
@@ -3669,7 +3691,11 @@
         </is>
       </c>
       <c r="Y31" s="11" t="n"/>
-      <c r="Z31" s="11" t="n"/>
+      <c r="Z31" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA31" s="11" t="n"/>
       <c r="AB31" s="14" t="inlineStr">
         <is>
@@ -3767,7 +3793,11 @@
         </is>
       </c>
       <c r="Y32" s="11" t="n"/>
-      <c r="Z32" s="11" t="n"/>
+      <c r="Z32" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA32" s="11" t="n"/>
       <c r="AB32" s="14" t="inlineStr">
         <is>
@@ -3865,7 +3895,11 @@
         </is>
       </c>
       <c r="Y33" s="11" t="n"/>
-      <c r="Z33" s="11" t="n"/>
+      <c r="Z33" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA33" s="11" t="n"/>
       <c r="AB33" s="14" t="inlineStr">
         <is>
@@ -3963,7 +3997,11 @@
         </is>
       </c>
       <c r="Y34" s="11" t="n"/>
-      <c r="Z34" s="11" t="n"/>
+      <c r="Z34" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA34" s="11" t="n"/>
       <c r="AB34" s="14" t="inlineStr">
         <is>
@@ -4061,7 +4099,11 @@
         </is>
       </c>
       <c r="Y35" s="11" t="n"/>
-      <c r="Z35" s="11" t="n"/>
+      <c r="Z35" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA35" s="11" t="n"/>
       <c r="AB35" s="14" t="inlineStr">
         <is>
@@ -4159,7 +4201,11 @@
         </is>
       </c>
       <c r="Y36" s="11" t="n"/>
-      <c r="Z36" s="11" t="n"/>
+      <c r="Z36" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA36" s="11" t="n"/>
       <c r="AB36" s="14" t="inlineStr">
         <is>
@@ -4191,7 +4237,7 @@
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F37" s="9" t="inlineStr">
@@ -4227,46 +4273,28 @@
         <v/>
       </c>
       <c r="P37" s="11" t="n"/>
-      <c r="Q37" s="12" t="n">
-        <v>372070</v>
-      </c>
+      <c r="Q37" s="12" t="n"/>
       <c r="R37" s="13">
         <f>IF(OR(Q37="",Q37=0,O37=""),"",O37/Q37)</f>
         <v/>
       </c>
-      <c r="S37" s="11" t="inlineStr">
-        <is>
-          <t>0.090</t>
-        </is>
-      </c>
-      <c r="T37" s="11" t="inlineStr">
-        <is>
-          <t>1100 (Single Family)</t>
-        </is>
-      </c>
+      <c r="S37" s="11" t="n"/>
+      <c r="T37" s="11" t="n"/>
       <c r="U37" s="11" t="n"/>
       <c r="V37" s="11" t="n"/>
-      <c r="W37" s="11" t="inlineStr">
-        <is>
-          <t>Massengill Josh (Jtwros)</t>
-        </is>
-      </c>
-      <c r="X37" s="11" t="inlineStr">
-        <is>
-          <t>12/08/2020 $282,000</t>
-        </is>
-      </c>
+      <c r="W37" s="11" t="n"/>
+      <c r="X37" s="11" t="inlineStr"/>
       <c r="Y37" s="11" t="n"/>
-      <c r="Z37" s="11" t="n"/>
+      <c r="Z37" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="AA37" s="11" t="n"/>
-      <c r="AB37" s="14" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
+      <c r="AB37" s="11" t="n"/>
       <c r="AC37" s="9" t="inlineStr">
         <is>
-          <t>608 Kingsmoor Drive Simpsonville, SC 29681 — 1100 (Single Family) — 0.090 ac (Autumn Trace). Record owner Massengill Josh (Jtwros). Last transfer 12/08/2020 for $282,000. County FMV $372,070.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>608 Kingsmoor Drive Simpsonville, SC 29681. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -11099,107 +11127,132 @@
   </sheetData>
   <autoFilter ref="A1:AC123"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB21" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB37" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y38" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y39" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y42" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y43" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y44" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y45" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y46" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y47" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y48" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y49" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y52" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y54" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y55" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y57" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y58" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y60" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y61" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y62" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y63" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y64" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y65" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y66" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y67" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y68" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y69" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y70" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y71" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y72" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y73" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y38" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y39" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y42" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y43" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y44" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y45" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y46" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y47" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y48" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y49" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y52" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y54" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y55" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y57" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y58" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y60" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y61" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y62" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y63" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y64" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y65" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y66" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y67" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y68" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y69" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y70" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y71" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y72" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y73" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId126"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
foreclosures: Greenville 9/8 Form 4 amounts (read by hand) + equity ranking
18 judgment totals loaded into the seed/state (extractedBy = manual), #6 and
#14 withdrawn; worklist regenerated with FMV−debt and a debt÷FMV read.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017rdAjmKGDVGAtDqQodYkcB
</commit_message>
<xml_diff>
--- a/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
+++ b/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
@@ -1705,7 +1705,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K10" s="12" t="n"/>
+      <c r="K10" s="12" t="n">
+        <v>94593</v>
+      </c>
       <c r="L10" s="10" t="n"/>
       <c r="M10" s="12" t="n"/>
       <c r="N10" s="11">
@@ -1746,7 +1748,11 @@
           <t>06/30/2006 $98,000</t>
         </is>
       </c>
-      <c r="Y10" s="11" t="n"/>
+      <c r="Y10" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z10" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -1760,7 +1766,7 @@
       </c>
       <c r="AC10" s="9" t="inlineStr">
         <is>
-          <t>9-A Stadium Drive Greenville, SC 29609 — 1100 (Single Family) — 0.520 ac. Record owner Walker Lonietta Y. Last transfer 06/30/2006 for $98,000. County FMV $218,570.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>9-A Stadium Drive Greenville, SC 29609 — 1100 (Single Family) — 0.520 ac. Record owner Walker Lonietta Y. Last transfer 06/30/2006 for $98,000. County FMV $218,570.00. Judgment $94,593.00. Debt is 43% of FMV — real equity, expect third-party bidding. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1813,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K11" s="12" t="n"/>
+      <c r="K11" s="12" t="n">
+        <v>331126</v>
+      </c>
       <c r="L11" s="10" t="n"/>
       <c r="M11" s="12" t="n"/>
       <c r="N11" s="11">
@@ -1848,7 +1856,11 @@
           <t>01/23/2024 $5</t>
         </is>
       </c>
-      <c r="Y11" s="11" t="n"/>
+      <c r="Y11" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z11" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -1862,7 +1874,7 @@
       </c>
       <c r="AC11" s="9" t="inlineStr">
         <is>
-          <t>304 Weddington Lane Simpsonville, SC 29681 — 1180 (Residential Vacant) — 0.150 ac (Linden Park). Record owner Key-Line Capital Investment Gr. Last transfer 01/23/2024 for $5. County FMV $95,000.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>304 Weddington Lane Simpsonville, SC 29681 — 1180 (Residential Vacant) — 0.150 ac (Linden Park). Record owner Key-Line Capital Investment Gr. Last transfer 01/23/2024 for $5. County FMV $95,000.00. Judgment $331,126.00. Debt exceeds FMV (349%) — plaintiff will likely take it back. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1921,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K12" s="12" t="n"/>
+      <c r="K12" s="12" t="n">
+        <v>482293</v>
+      </c>
       <c r="L12" s="10" t="n"/>
       <c r="M12" s="12" t="n"/>
       <c r="N12" s="11">
@@ -1950,7 +1964,11 @@
           <t>11/13/2023 $400,000</t>
         </is>
       </c>
-      <c r="Y12" s="11" t="n"/>
+      <c r="Y12" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z12" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -1964,7 +1982,7 @@
       </c>
       <c r="AC12" s="9" t="inlineStr">
         <is>
-          <t>608 Rhett Street Greenville, SC 29601 — 1100 (Single Family) — 0.100 ac. Record owner Vswc Llc. Last transfer 11/13/2023 for $400,000. County FMV $392,670.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>608 Rhett Street Greenville, SC 29601 — 1100 (Single Family) — 0.100 ac. Record owner Vswc Llc. Last transfer 11/13/2023 for $400,000. County FMV $392,670.00. Judgment $482,293.00. Debt exceeds FMV (123%) — plaintiff will likely take it back. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2029,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K13" s="12" t="n"/>
+      <c r="K13" s="12" t="n">
+        <v>179057</v>
+      </c>
       <c r="L13" s="10" t="n"/>
       <c r="M13" s="12" t="n"/>
       <c r="N13" s="11">
@@ -2052,7 +2072,11 @@
           <t>09/29/2020 $179,000</t>
         </is>
       </c>
-      <c r="Y13" s="11" t="n"/>
+      <c r="Y13" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z13" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2066,7 +2090,7 @@
       </c>
       <c r="AC13" s="9" t="inlineStr">
         <is>
-          <t>4 Point Hope Court Greenville, SC 29605 — 1100 (Single Family) (Oak Knoll). Record owner Culpepper-Booker Sharon Diane. Last transfer 09/29/2020 for $179,000. County FMV $235,180.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>4 Point Hope Court Greenville, SC 29605 — 1100 (Single Family) (Oak Knoll). Record owner Culpepper-Booker Sharon Diane. Last transfer 09/29/2020 for $179,000. County FMV $235,180.00. Judgment $179,057.00. Debt is 76% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2113,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -2146,7 +2170,7 @@
       <c r="AB14" s="11" t="n"/>
       <c r="AC14" s="9" t="inlineStr">
         <is>
-          <t>110 Water Reach Lane Simpsonville, SC 29681. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>110 Water Reach Lane Simpsonville, SC 29681. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2297,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K16" s="12" t="n"/>
+      <c r="K16" s="12" t="n">
+        <v>68468.05</v>
+      </c>
       <c r="L16" s="10" t="n"/>
       <c r="M16" s="12" t="n"/>
       <c r="N16" s="11">
@@ -2314,7 +2340,11 @@
           <t>05/20/2014 $132,500</t>
         </is>
       </c>
-      <c r="Y16" s="11" t="n"/>
+      <c r="Y16" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z16" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2328,7 +2358,7 @@
       </c>
       <c r="AC16" s="9" t="inlineStr">
         <is>
-          <t>39B W Golden Strip Drive Mauldin, SC 29662 — 1100 (Single Family) — 0.340 ac. Record owner Ladson Alice D (card is for 39 W GOLDEN STRIP DR — unit letter not on file, verify). Last transfer 05/20/2014 for $132,500. County FMV $244,440.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>39B W Golden Strip Drive Mauldin, SC 29662 — 1100 (Single Family) — 0.340 ac. Record owner Ladson Alice D (card is for 39 W GOLDEN STRIP DR — unit letter not on file, verify). Last transfer 05/20/2014 for $132,500. County FMV $244,440.00. Judgment $68,468.05. Debt is 28% of FMV — real equity, expect third-party bidding. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2405,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K17" s="12" t="n"/>
+      <c r="K17" s="12" t="n">
+        <v>279737</v>
+      </c>
       <c r="L17" s="10" t="n"/>
       <c r="M17" s="12" t="n"/>
       <c r="N17" s="11">
@@ -2416,7 +2448,11 @@
           <t>05/11/2023 $262,999</t>
         </is>
       </c>
-      <c r="Y17" s="11" t="n"/>
+      <c r="Y17" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z17" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2430,7 +2466,7 @@
       </c>
       <c r="AC17" s="9" t="inlineStr">
         <is>
-          <t>15 Fennec Drive Fountain Inn, SC 29644 — 1100 (Single Family) (Fox Tail Cottages). Record owner Roane Brandon Andre. Last transfer 05/11/2023 for $262,999. County FMV $289,220.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>15 Fennec Drive Fountain Inn, SC 29644 — 1100 (Single Family) (Fox Tail Cottages). Record owner Roane Brandon Andre. Last transfer 05/11/2023 for $262,999. County FMV $289,220.00. Judgment $279,737.00. Debt is 97% of FMV — thin margin. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2513,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K18" s="12" t="n"/>
+      <c r="K18" s="12" t="n">
+        <v>254440</v>
+      </c>
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="12" t="n"/>
       <c r="N18" s="11">
@@ -2518,7 +2556,11 @@
           <t>01/17/2024 $222,500</t>
         </is>
       </c>
-      <c r="Y18" s="11" t="n"/>
+      <c r="Y18" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z18" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2532,7 +2574,7 @@
       </c>
       <c r="AC18" s="9" t="inlineStr">
         <is>
-          <t>104 Pine Needle Road Piedmont, SC 29673 — 1100 (Single Family) (Pine Shadows). Record owner Rhodes Ashley. Last transfer 01/17/2024 for $222,500. County FMV $212,830.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>104 Pine Needle Road Piedmont, SC 29673 — 1100 (Single Family) (Pine Shadows). Record owner Rhodes Ashley. Last transfer 01/17/2024 for $222,500. County FMV $212,830.00. Judgment $254,440.00. Debt exceeds FMV (120%) — plaintiff will likely take it back. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2579,7 +2621,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K19" s="12" t="n"/>
+      <c r="K19" s="12" t="n">
+        <v>906485</v>
+      </c>
       <c r="L19" s="10" t="n"/>
       <c r="M19" s="12" t="n"/>
       <c r="N19" s="11">
@@ -2602,7 +2646,11 @@
       <c r="V19" s="11" t="n"/>
       <c r="W19" s="11" t="n"/>
       <c r="X19" s="11" t="inlineStr"/>
-      <c r="Y19" s="11" t="n"/>
+      <c r="Y19" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z19" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2612,7 +2660,7 @@
       <c r="AB19" s="11" t="n"/>
       <c r="AC19" s="9" t="inlineStr">
         <is>
-          <t>402 Sienna Drive Greenville, SC 29609. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>402 Sienna Drive Greenville, SC 29609. Judgment $906,485.00. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2707,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K20" s="12" t="n"/>
+      <c r="K20" s="12" t="n">
+        <v>269097</v>
+      </c>
       <c r="L20" s="10" t="n"/>
       <c r="M20" s="12" t="n"/>
       <c r="N20" s="11">
@@ -2700,7 +2750,11 @@
           <t>11/15/2023 $244,900</t>
         </is>
       </c>
-      <c r="Y20" s="11" t="n"/>
+      <c r="Y20" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z20" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2714,7 +2768,7 @@
       </c>
       <c r="AC20" s="9" t="inlineStr">
         <is>
-          <t>3 Black Oak Court Simpsonville, SC 29680 — 1100 (Single Family) (Standing Springs Estate). Record owner Harley Maria. Last transfer 11/15/2023 for $244,900. County FMV $278,430.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>3 Black Oak Court Simpsonville, SC 29680 — 1100 (Single Family) (Standing Springs Estate). Record owner Harley Maria. Last transfer 11/15/2023 for $244,900. County FMV $278,430.00. Judgment $269,097.00. Debt is 97% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2871,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -2896,7 +2950,7 @@
       </c>
       <c r="AC22" s="9" t="inlineStr">
         <is>
-          <t>1904 Lake Cunningham Road Greer, SC 29651 — 1170 (MH w/ land) (Cunningham Downs). Record owner Morales-Greene Emilia. Last transfer 06/27/2025. County FMV $410,930.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>1904 Lake Cunningham Road Greer, SC 29651 — 1170 (MH w/ land) (Cunningham Downs). Record owner Morales-Greene Emilia. Last transfer 06/27/2025. County FMV $410,930.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3077,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K24" s="12" t="n"/>
+      <c r="K24" s="12" t="n">
+        <v>107886</v>
+      </c>
       <c r="L24" s="10" t="n"/>
       <c r="M24" s="12" t="n"/>
       <c r="N24" s="11">
@@ -3064,7 +3120,11 @@
           <t>12/01/2009 $10</t>
         </is>
       </c>
-      <c r="Y24" s="11" t="n"/>
+      <c r="Y24" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z24" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3078,7 +3138,7 @@
       </c>
       <c r="AC24" s="9" t="inlineStr">
         <is>
-          <t>1406 Winding Way Taylors, SC 29687 — 1100 (Single Family) (Peppertree). Record owner Dixon Sue Ann. Last transfer 12/01/2009 for $10. County FMV $254,770.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>1406 Winding Way Taylors, SC 29687 — 1100 (Single Family) (Peppertree). Record owner Dixon Sue Ann. Last transfer 12/01/2009 for $10. County FMV $254,770.00. Judgment $107,886.00. Debt is 42% of FMV — real equity, expect third-party bidding. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3265,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K26" s="12" t="n"/>
+      <c r="K26" s="12" t="n">
+        <v>408231</v>
+      </c>
       <c r="L26" s="10" t="n"/>
       <c r="M26" s="12" t="n"/>
       <c r="N26" s="11">
@@ -3246,7 +3308,11 @@
           <t>04/11/2022 $389,900</t>
         </is>
       </c>
-      <c r="Y26" s="11" t="n"/>
+      <c r="Y26" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z26" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3260,7 +3326,7 @@
       </c>
       <c r="AC26" s="9" t="inlineStr">
         <is>
-          <t>104 Oak Forest Drive Greer, SC 29650 — 1100 (Single Family). Record owner Thompson Chad. Last transfer 04/11/2022 for $389,900. County FMV $522,800.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>104 Oak Forest Drive Greer, SC 29650 — 1100 (Single Family). Record owner Thompson Chad. Last transfer 04/11/2022 for $389,900. County FMV $522,800.00. Judgment $408,231.00. Debt is 78% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3453,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K28" s="12" t="n"/>
+      <c r="K28" s="12" t="n">
+        <v>4572030.1</v>
+      </c>
       <c r="L28" s="10" t="n"/>
       <c r="M28" s="12" t="n"/>
       <c r="N28" s="11">
@@ -3428,7 +3496,11 @@
           <t>12/16/2019</t>
         </is>
       </c>
-      <c r="Y28" s="11" t="n"/>
+      <c r="Y28" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z28" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3442,7 +3514,7 @@
       </c>
       <c r="AC28" s="9" t="inlineStr">
         <is>
-          <t>100 N. Markley St. Greenville, SC 29601 — 6800 (Commercial Vacant ) — 0.910 ac. Record owner Greenville Hkw Llc. Last transfer 12/16/2019. County FMV $2,973,000.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>100 N. Markley St. Greenville, SC 29601 — 6800 (Commercial Vacant ) — 0.910 ac. Record owner Greenville Hkw Llc. Last transfer 12/16/2019. County FMV $2,973,000.00. Judgment $4,572,030.10. Debt exceeds FMV (154%) — plaintiff will likely take it back. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3721,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K31" s="12" t="n"/>
+      <c r="K31" s="12" t="n">
+        <v>153841.1</v>
+      </c>
       <c r="L31" s="10" t="n"/>
       <c r="M31" s="12" t="n"/>
       <c r="N31" s="11">
@@ -3690,7 +3764,11 @@
           <t>11/15/2004 $105,000</t>
         </is>
       </c>
-      <c r="Y31" s="11" t="n"/>
+      <c r="Y31" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z31" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3704,7 +3782,7 @@
       </c>
       <c r="AC31" s="9" t="inlineStr">
         <is>
-          <t>304 Glenlea Ln Greenville, SC 29617 — 1100 (Single Family) — 0.120 ac (The Village At Glenlea). Record owner Staton Beverly. Last transfer 11/15/2004 for $105,000. County FMV $224,920.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>304 Glenlea Ln Greenville, SC 29617 — 1100 (Single Family) — 0.120 ac (The Village At Glenlea). Record owner Staton Beverly. Last transfer 11/15/2004 for $105,000. County FMV $224,920.00. Judgment $153,841.10. Debt is 68% of FMV — real equity, expect third-party bidding. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3829,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K32" s="12" t="n"/>
+      <c r="K32" s="12" t="n">
+        <v>246879.23</v>
+      </c>
       <c r="L32" s="10" t="n"/>
       <c r="M32" s="12" t="n"/>
       <c r="N32" s="11">
@@ -3792,7 +3872,11 @@
           <t>10/05/2021 $100,000</t>
         </is>
       </c>
-      <c r="Y32" s="11" t="n"/>
+      <c r="Y32" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z32" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3806,7 +3890,7 @@
       </c>
       <c r="AC32" s="9" t="inlineStr">
         <is>
-          <t>71 Dorsey Avenue Greenville, SC 29611 — 1100 (Single Family) — 0.210 ac (Abney Mills). Record owner Vswc Llc. Last transfer 10/05/2021 for $100,000. County FMV $246,770.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>71 Dorsey Avenue Greenville, SC 29611 — 1100 (Single Family) — 0.210 ac (Abney Mills). Record owner Vswc Llc. Last transfer 10/05/2021 for $100,000. County FMV $246,770.00. Judgment $246,879.23. Debt exceeds FMV (100%) — plaintiff will likely take it back. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3937,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K33" s="12" t="n"/>
+      <c r="K33" s="12" t="n">
+        <v>159379.2</v>
+      </c>
       <c r="L33" s="10" t="n"/>
       <c r="M33" s="12" t="n"/>
       <c r="N33" s="11">
@@ -3894,7 +3980,11 @@
           <t>05/21/2020 $10</t>
         </is>
       </c>
-      <c r="Y33" s="11" t="n"/>
+      <c r="Y33" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z33" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3908,7 +3998,7 @@
       </c>
       <c r="AC33" s="9" t="inlineStr">
         <is>
-          <t>37 Ross Street Greenville, SC 29611 — 1100 (Single Family). Record owner Vswc Llc. Last transfer 05/21/2020 for $10. County FMV $183,180.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>37 Ross Street Greenville, SC 29611 — 1100 (Single Family). Record owner Vswc Llc. Last transfer 05/21/2020 for $10. County FMV $183,180.00. Judgment $159,379.20. Debt is 87% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3955,7 +4045,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K34" s="12" t="n"/>
+      <c r="K34" s="12" t="n">
+        <v>219174.3</v>
+      </c>
       <c r="L34" s="10" t="n"/>
       <c r="M34" s="12" t="n"/>
       <c r="N34" s="11">
@@ -3996,7 +4088,11 @@
           <t>08/12/2022 $235,000</t>
         </is>
       </c>
-      <c r="Y34" s="11" t="n"/>
+      <c r="Y34" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z34" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -4010,7 +4106,7 @@
       </c>
       <c r="AC34" s="9" t="inlineStr">
         <is>
-          <t>11 Charing Cross Road Taylors, SC 29687 — 1100 (Single Family) (Brookwood Forest). Record owner Grm Properties Of South Caroli. Last transfer 08/12/2022 for $235,000. County FMV $267,670.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>11 Charing Cross Road Taylors, SC 29687 — 1100 (Single Family) (Brookwood Forest). Record owner Grm Properties Of South Caroli. Last transfer 08/12/2022 for $235,000. County FMV $267,670.00. Judgment $219,174.30. Debt is 82% of FMV — thin margin. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4153,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K35" s="12" t="n"/>
+      <c r="K35" s="12" t="n">
+        <v>301030.64</v>
+      </c>
       <c r="L35" s="10" t="n"/>
       <c r="M35" s="12" t="n"/>
       <c r="N35" s="11">
@@ -4098,7 +4196,11 @@
           <t>05/02/2022 $130,000</t>
         </is>
       </c>
-      <c r="Y35" s="11" t="n"/>
+      <c r="Y35" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z35" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -4112,7 +4214,7 @@
       </c>
       <c r="AC35" s="9" t="inlineStr">
         <is>
-          <t>2501 Poinsett Highway Greenville, SC 29609 — 1100 (Single Family). Record owner 2501 Poinsette Llc. Last transfer 05/02/2022 for $130,000. County FMV $306,870.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>2501 Poinsett Highway Greenville, SC 29609 — 1100 (Single Family). Record owner 2501 Poinsette Llc. Last transfer 05/02/2022 for $130,000. County FMV $306,870.00. Judgment $301,030.64. Debt is 98% of FMV — thin margin. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4261,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K36" s="12" t="n"/>
+      <c r="K36" s="12" t="n">
+        <v>221056.42</v>
+      </c>
       <c r="L36" s="10" t="n"/>
       <c r="M36" s="12" t="n"/>
       <c r="N36" s="11">
@@ -4200,7 +4304,11 @@
           <t>05/16/2023 $249,900</t>
         </is>
       </c>
-      <c r="Y36" s="11" t="n"/>
+      <c r="Y36" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z36" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -4214,7 +4322,7 @@
       </c>
       <c r="AC36" s="9" t="inlineStr">
         <is>
-          <t>202 Port Road Greenville, SC 29617 — 1100 (Single Family) — 0.590 ac (River Valley). Record owner Green Ant Llc. Last transfer 05/16/2023 for $249,900. County FMV $249,890.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>202 Port Road Greenville, SC 29617 — 1100 (Single Family) — 0.590 ac (River Valley). Record owner Green Ant Llc. Last transfer 05/16/2023 for $249,900. County FMV $249,890.00. Judgment $221,056.42. Debt is 88% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -11128,131 +11236,149 @@
   <autoFilter ref="A1:AC123"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y38" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y39" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y42" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y43" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y44" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y45" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y46" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y47" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y48" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y49" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y52" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y54" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y55" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y57" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y58" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y60" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y61" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y62" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y63" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y64" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y65" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y66" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y67" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y68" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y69" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y70" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y71" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y72" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y73" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y24" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y26" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y28" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y31" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y32" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y33" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y34" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y35" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y36" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y38" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y39" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y42" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y43" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y44" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y45" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y46" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y47" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y48" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y49" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y52" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y54" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y55" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y57" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y58" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y60" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y61" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y62" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y63" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y64" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y65" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y66" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y67" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y68" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y69" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y70" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y71" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y72" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y73" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId144"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Foreclosures: Greenville 9/8 Form 4 amounts + equity ranking (#75)
18 judgment totals loaded into the seed/state (extractedBy = manual), #6 and
#14 withdrawn; worklist regenerated with FMV−debt and a debt÷FMV read.


Claude-Session: https://claude.ai/code/session_017rdAjmKGDVGAtDqQodYkcB

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
+++ b/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
@@ -1705,7 +1705,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K10" s="12" t="n"/>
+      <c r="K10" s="12" t="n">
+        <v>94593</v>
+      </c>
       <c r="L10" s="10" t="n"/>
       <c r="M10" s="12" t="n"/>
       <c r="N10" s="11">
@@ -1746,7 +1748,11 @@
           <t>06/30/2006 $98,000</t>
         </is>
       </c>
-      <c r="Y10" s="11" t="n"/>
+      <c r="Y10" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z10" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -1760,7 +1766,7 @@
       </c>
       <c r="AC10" s="9" t="inlineStr">
         <is>
-          <t>9-A Stadium Drive Greenville, SC 29609 — 1100 (Single Family) — 0.520 ac. Record owner Walker Lonietta Y. Last transfer 06/30/2006 for $98,000. County FMV $218,570.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>9-A Stadium Drive Greenville, SC 29609 — 1100 (Single Family) — 0.520 ac. Record owner Walker Lonietta Y. Last transfer 06/30/2006 for $98,000. County FMV $218,570.00. Judgment $94,593.00. Debt is 43% of FMV — real equity, expect third-party bidding. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -1807,7 +1813,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K11" s="12" t="n"/>
+      <c r="K11" s="12" t="n">
+        <v>331126</v>
+      </c>
       <c r="L11" s="10" t="n"/>
       <c r="M11" s="12" t="n"/>
       <c r="N11" s="11">
@@ -1848,7 +1856,11 @@
           <t>01/23/2024 $5</t>
         </is>
       </c>
-      <c r="Y11" s="11" t="n"/>
+      <c r="Y11" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z11" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -1862,7 +1874,7 @@
       </c>
       <c r="AC11" s="9" t="inlineStr">
         <is>
-          <t>304 Weddington Lane Simpsonville, SC 29681 — 1180 (Residential Vacant) — 0.150 ac (Linden Park). Record owner Key-Line Capital Investment Gr. Last transfer 01/23/2024 for $5. County FMV $95,000.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>304 Weddington Lane Simpsonville, SC 29681 — 1180 (Residential Vacant) — 0.150 ac (Linden Park). Record owner Key-Line Capital Investment Gr. Last transfer 01/23/2024 for $5. County FMV $95,000.00. Judgment $331,126.00. Debt exceeds FMV (349%) — plaintiff will likely take it back. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1921,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K12" s="12" t="n"/>
+      <c r="K12" s="12" t="n">
+        <v>482293</v>
+      </c>
       <c r="L12" s="10" t="n"/>
       <c r="M12" s="12" t="n"/>
       <c r="N12" s="11">
@@ -1950,7 +1964,11 @@
           <t>11/13/2023 $400,000</t>
         </is>
       </c>
-      <c r="Y12" s="11" t="n"/>
+      <c r="Y12" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z12" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -1964,7 +1982,7 @@
       </c>
       <c r="AC12" s="9" t="inlineStr">
         <is>
-          <t>608 Rhett Street Greenville, SC 29601 — 1100 (Single Family) — 0.100 ac. Record owner Vswc Llc. Last transfer 11/13/2023 for $400,000. County FMV $392,670.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>608 Rhett Street Greenville, SC 29601 — 1100 (Single Family) — 0.100 ac. Record owner Vswc Llc. Last transfer 11/13/2023 for $400,000. County FMV $392,670.00. Judgment $482,293.00. Debt exceeds FMV (123%) — plaintiff will likely take it back. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2029,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K13" s="12" t="n"/>
+      <c r="K13" s="12" t="n">
+        <v>179057</v>
+      </c>
       <c r="L13" s="10" t="n"/>
       <c r="M13" s="12" t="n"/>
       <c r="N13" s="11">
@@ -2052,7 +2072,11 @@
           <t>09/29/2020 $179,000</t>
         </is>
       </c>
-      <c r="Y13" s="11" t="n"/>
+      <c r="Y13" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z13" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2066,7 +2090,7 @@
       </c>
       <c r="AC13" s="9" t="inlineStr">
         <is>
-          <t>4 Point Hope Court Greenville, SC 29605 — 1100 (Single Family) (Oak Knoll). Record owner Culpepper-Booker Sharon Diane. Last transfer 09/29/2020 for $179,000. County FMV $235,180.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>4 Point Hope Court Greenville, SC 29605 — 1100 (Single Family) (Oak Knoll). Record owner Culpepper-Booker Sharon Diane. Last transfer 09/29/2020 for $179,000. County FMV $235,180.00. Judgment $179,057.00. Debt is 76% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2113,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -2146,7 +2170,7 @@
       <c r="AB14" s="11" t="n"/>
       <c r="AC14" s="9" t="inlineStr">
         <is>
-          <t>110 Water Reach Lane Simpsonville, SC 29681. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>110 Water Reach Lane Simpsonville, SC 29681. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -2273,7 +2297,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K16" s="12" t="n"/>
+      <c r="K16" s="12" t="n">
+        <v>68468.05</v>
+      </c>
       <c r="L16" s="10" t="n"/>
       <c r="M16" s="12" t="n"/>
       <c r="N16" s="11">
@@ -2314,7 +2340,11 @@
           <t>05/20/2014 $132,500</t>
         </is>
       </c>
-      <c r="Y16" s="11" t="n"/>
+      <c r="Y16" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z16" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2328,7 +2358,7 @@
       </c>
       <c r="AC16" s="9" t="inlineStr">
         <is>
-          <t>39B W Golden Strip Drive Mauldin, SC 29662 — 1100 (Single Family) — 0.340 ac. Record owner Ladson Alice D (card is for 39 W GOLDEN STRIP DR — unit letter not on file, verify). Last transfer 05/20/2014 for $132,500. County FMV $244,440.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>39B W Golden Strip Drive Mauldin, SC 29662 — 1100 (Single Family) — 0.340 ac. Record owner Ladson Alice D (card is for 39 W GOLDEN STRIP DR — unit letter not on file, verify). Last transfer 05/20/2014 for $132,500. County FMV $244,440.00. Judgment $68,468.05. Debt is 28% of FMV — real equity, expect third-party bidding. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2405,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K17" s="12" t="n"/>
+      <c r="K17" s="12" t="n">
+        <v>279737</v>
+      </c>
       <c r="L17" s="10" t="n"/>
       <c r="M17" s="12" t="n"/>
       <c r="N17" s="11">
@@ -2416,7 +2448,11 @@
           <t>05/11/2023 $262,999</t>
         </is>
       </c>
-      <c r="Y17" s="11" t="n"/>
+      <c r="Y17" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z17" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2430,7 +2466,7 @@
       </c>
       <c r="AC17" s="9" t="inlineStr">
         <is>
-          <t>15 Fennec Drive Fountain Inn, SC 29644 — 1100 (Single Family) (Fox Tail Cottages). Record owner Roane Brandon Andre. Last transfer 05/11/2023 for $262,999. County FMV $289,220.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>15 Fennec Drive Fountain Inn, SC 29644 — 1100 (Single Family) (Fox Tail Cottages). Record owner Roane Brandon Andre. Last transfer 05/11/2023 for $262,999. County FMV $289,220.00. Judgment $279,737.00. Debt is 97% of FMV — thin margin. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -2477,7 +2513,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K18" s="12" t="n"/>
+      <c r="K18" s="12" t="n">
+        <v>254440</v>
+      </c>
       <c r="L18" s="10" t="n"/>
       <c r="M18" s="12" t="n"/>
       <c r="N18" s="11">
@@ -2518,7 +2556,11 @@
           <t>01/17/2024 $222,500</t>
         </is>
       </c>
-      <c r="Y18" s="11" t="n"/>
+      <c r="Y18" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z18" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2532,7 +2574,7 @@
       </c>
       <c r="AC18" s="9" t="inlineStr">
         <is>
-          <t>104 Pine Needle Road Piedmont, SC 29673 — 1100 (Single Family) (Pine Shadows). Record owner Rhodes Ashley. Last transfer 01/17/2024 for $222,500. County FMV $212,830.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>104 Pine Needle Road Piedmont, SC 29673 — 1100 (Single Family) (Pine Shadows). Record owner Rhodes Ashley. Last transfer 01/17/2024 for $222,500. County FMV $212,830.00. Judgment $254,440.00. Debt exceeds FMV (120%) — plaintiff will likely take it back. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2579,7 +2621,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K19" s="12" t="n"/>
+      <c r="K19" s="12" t="n">
+        <v>906485</v>
+      </c>
       <c r="L19" s="10" t="n"/>
       <c r="M19" s="12" t="n"/>
       <c r="N19" s="11">
@@ -2602,7 +2646,11 @@
       <c r="V19" s="11" t="n"/>
       <c r="W19" s="11" t="n"/>
       <c r="X19" s="11" t="inlineStr"/>
-      <c r="Y19" s="11" t="n"/>
+      <c r="Y19" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z19" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2612,7 +2660,7 @@
       <c r="AB19" s="11" t="n"/>
       <c r="AC19" s="9" t="inlineStr">
         <is>
-          <t>402 Sienna Drive Greenville, SC 29609. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>402 Sienna Drive Greenville, SC 29609. Judgment $906,485.00. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2659,7 +2707,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K20" s="12" t="n"/>
+      <c r="K20" s="12" t="n">
+        <v>269097</v>
+      </c>
       <c r="L20" s="10" t="n"/>
       <c r="M20" s="12" t="n"/>
       <c r="N20" s="11">
@@ -2700,7 +2750,11 @@
           <t>11/15/2023 $244,900</t>
         </is>
       </c>
-      <c r="Y20" s="11" t="n"/>
+      <c r="Y20" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z20" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -2714,7 +2768,7 @@
       </c>
       <c r="AC20" s="9" t="inlineStr">
         <is>
-          <t>3 Black Oak Court Simpsonville, SC 29680 — 1100 (Single Family) (Standing Springs Estate). Record owner Harley Maria. Last transfer 11/15/2023 for $244,900. County FMV $278,430.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>3 Black Oak Court Simpsonville, SC 29680 — 1100 (Single Family) (Standing Springs Estate). Record owner Harley Maria. Last transfer 11/15/2023 for $244,900. County FMV $278,430.00. Judgment $269,097.00. Debt is 97% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2871,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>scheduled</t>
+          <t>withdrawn</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -2896,7 +2950,7 @@
       </c>
       <c r="AC22" s="9" t="inlineStr">
         <is>
-          <t>1904 Lake Cunningham Road Greer, SC 29651 — 1170 (MH w/ land) (Cunningham Downs). Record owner Morales-Greene Emilia. Last transfer 06/27/2025. County FMV $410,930.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>1904 Lake Cunningham Road Greer, SC 29651 — 1170 (MH w/ land) (Cunningham Downs). Record owner Morales-Greene Emilia. Last transfer 06/27/2025. County FMV $410,930.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day. STATUS: WITHDRAWN.</t>
         </is>
       </c>
     </row>
@@ -3023,7 +3077,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K24" s="12" t="n"/>
+      <c r="K24" s="12" t="n">
+        <v>107886</v>
+      </c>
       <c r="L24" s="10" t="n"/>
       <c r="M24" s="12" t="n"/>
       <c r="N24" s="11">
@@ -3064,7 +3120,11 @@
           <t>12/01/2009 $10</t>
         </is>
       </c>
-      <c r="Y24" s="11" t="n"/>
+      <c r="Y24" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z24" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3078,7 +3138,7 @@
       </c>
       <c r="AC24" s="9" t="inlineStr">
         <is>
-          <t>1406 Winding Way Taylors, SC 29687 — 1100 (Single Family) (Peppertree). Record owner Dixon Sue Ann. Last transfer 12/01/2009 for $10. County FMV $254,770.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>1406 Winding Way Taylors, SC 29687 — 1100 (Single Family) (Peppertree). Record owner Dixon Sue Ann. Last transfer 12/01/2009 for $10. County FMV $254,770.00. Judgment $107,886.00. Debt is 42% of FMV — real equity, expect third-party bidding. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -3205,7 +3265,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K26" s="12" t="n"/>
+      <c r="K26" s="12" t="n">
+        <v>408231</v>
+      </c>
       <c r="L26" s="10" t="n"/>
       <c r="M26" s="12" t="n"/>
       <c r="N26" s="11">
@@ -3246,7 +3308,11 @@
           <t>04/11/2022 $389,900</t>
         </is>
       </c>
-      <c r="Y26" s="11" t="n"/>
+      <c r="Y26" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z26" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3260,7 +3326,7 @@
       </c>
       <c r="AC26" s="9" t="inlineStr">
         <is>
-          <t>104 Oak Forest Drive Greer, SC 29650 — 1100 (Single Family). Record owner Thompson Chad. Last transfer 04/11/2022 for $389,900. County FMV $522,800.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>104 Oak Forest Drive Greer, SC 29650 — 1100 (Single Family). Record owner Thompson Chad. Last transfer 04/11/2022 for $389,900. County FMV $522,800.00. Judgment $408,231.00. Debt is 78% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3387,7 +3453,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K28" s="12" t="n"/>
+      <c r="K28" s="12" t="n">
+        <v>4572030.1</v>
+      </c>
       <c r="L28" s="10" t="n"/>
       <c r="M28" s="12" t="n"/>
       <c r="N28" s="11">
@@ -3428,7 +3496,11 @@
           <t>12/16/2019</t>
         </is>
       </c>
-      <c r="Y28" s="11" t="n"/>
+      <c r="Y28" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z28" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3442,7 +3514,7 @@
       </c>
       <c r="AC28" s="9" t="inlineStr">
         <is>
-          <t>100 N. Markley St. Greenville, SC 29601 — 6800 (Commercial Vacant ) — 0.910 ac. Record owner Greenville Hkw Llc. Last transfer 12/16/2019. County FMV $2,973,000.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>100 N. Markley St. Greenville, SC 29601 — 6800 (Commercial Vacant ) — 0.910 ac. Record owner Greenville Hkw Llc. Last transfer 12/16/2019. County FMV $2,973,000.00. Judgment $4,572,030.10. Debt exceeds FMV (154%) — plaintiff will likely take it back. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3649,7 +3721,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K31" s="12" t="n"/>
+      <c r="K31" s="12" t="n">
+        <v>153841.1</v>
+      </c>
       <c r="L31" s="10" t="n"/>
       <c r="M31" s="12" t="n"/>
       <c r="N31" s="11">
@@ -3690,7 +3764,11 @@
           <t>11/15/2004 $105,000</t>
         </is>
       </c>
-      <c r="Y31" s="11" t="n"/>
+      <c r="Y31" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z31" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3704,7 +3782,7 @@
       </c>
       <c r="AC31" s="9" t="inlineStr">
         <is>
-          <t>304 Glenlea Ln Greenville, SC 29617 — 1100 (Single Family) — 0.120 ac (The Village At Glenlea). Record owner Staton Beverly. Last transfer 11/15/2004 for $105,000. County FMV $224,920.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>304 Glenlea Ln Greenville, SC 29617 — 1100 (Single Family) — 0.120 ac (The Village At Glenlea). Record owner Staton Beverly. Last transfer 11/15/2004 for $105,000. County FMV $224,920.00. Judgment $153,841.10. Debt is 68% of FMV — real equity, expect third-party bidding. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3829,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K32" s="12" t="n"/>
+      <c r="K32" s="12" t="n">
+        <v>246879.23</v>
+      </c>
       <c r="L32" s="10" t="n"/>
       <c r="M32" s="12" t="n"/>
       <c r="N32" s="11">
@@ -3792,7 +3872,11 @@
           <t>10/05/2021 $100,000</t>
         </is>
       </c>
-      <c r="Y32" s="11" t="n"/>
+      <c r="Y32" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z32" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3806,7 +3890,7 @@
       </c>
       <c r="AC32" s="9" t="inlineStr">
         <is>
-          <t>71 Dorsey Avenue Greenville, SC 29611 — 1100 (Single Family) — 0.210 ac (Abney Mills). Record owner Vswc Llc. Last transfer 10/05/2021 for $100,000. County FMV $246,770.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>71 Dorsey Avenue Greenville, SC 29611 — 1100 (Single Family) — 0.210 ac (Abney Mills). Record owner Vswc Llc. Last transfer 10/05/2021 for $100,000. County FMV $246,770.00. Judgment $246,879.23. Debt exceeds FMV (100%) — plaintiff will likely take it back. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3937,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K33" s="12" t="n"/>
+      <c r="K33" s="12" t="n">
+        <v>159379.2</v>
+      </c>
       <c r="L33" s="10" t="n"/>
       <c r="M33" s="12" t="n"/>
       <c r="N33" s="11">
@@ -3894,7 +3980,11 @@
           <t>05/21/2020 $10</t>
         </is>
       </c>
-      <c r="Y33" s="11" t="n"/>
+      <c r="Y33" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z33" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -3908,7 +3998,7 @@
       </c>
       <c r="AC33" s="9" t="inlineStr">
         <is>
-          <t>37 Ross Street Greenville, SC 29611 — 1100 (Single Family). Record owner Vswc Llc. Last transfer 05/21/2020 for $10. County FMV $183,180.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>37 Ross Street Greenville, SC 29611 — 1100 (Single Family). Record owner Vswc Llc. Last transfer 05/21/2020 for $10. County FMV $183,180.00. Judgment $159,379.20. Debt is 87% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -3955,7 +4045,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K34" s="12" t="n"/>
+      <c r="K34" s="12" t="n">
+        <v>219174.3</v>
+      </c>
       <c r="L34" s="10" t="n"/>
       <c r="M34" s="12" t="n"/>
       <c r="N34" s="11">
@@ -3996,7 +4088,11 @@
           <t>08/12/2022 $235,000</t>
         </is>
       </c>
-      <c r="Y34" s="11" t="n"/>
+      <c r="Y34" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z34" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -4010,7 +4106,7 @@
       </c>
       <c r="AC34" s="9" t="inlineStr">
         <is>
-          <t>11 Charing Cross Road Taylors, SC 29687 — 1100 (Single Family) (Brookwood Forest). Record owner Grm Properties Of South Caroli. Last transfer 08/12/2022 for $235,000. County FMV $267,670.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>11 Charing Cross Road Taylors, SC 29687 — 1100 (Single Family) (Brookwood Forest). Record owner Grm Properties Of South Caroli. Last transfer 08/12/2022 for $235,000. County FMV $267,670.00. Judgment $219,174.30. Debt is 82% of FMV — thin margin. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -4057,7 +4153,9 @@
           <t>demanded</t>
         </is>
       </c>
-      <c r="K35" s="12" t="n"/>
+      <c r="K35" s="12" t="n">
+        <v>301030.64</v>
+      </c>
       <c r="L35" s="10" t="n"/>
       <c r="M35" s="12" t="n"/>
       <c r="N35" s="11">
@@ -4098,7 +4196,11 @@
           <t>05/02/2022 $130,000</t>
         </is>
       </c>
-      <c r="Y35" s="11" t="n"/>
+      <c r="Y35" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z35" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -4112,7 +4214,7 @@
       </c>
       <c r="AC35" s="9" t="inlineStr">
         <is>
-          <t>2501 Poinsett Highway Greenville, SC 29609 — 1100 (Single Family). Record owner 2501 Poinsette Llc. Last transfer 05/02/2022 for $130,000. County FMV $306,870.00. Judgment $ not pulled yet (needs the PC run). DEFICIENCY DEMANDED — open 30 days.</t>
+          <t>2501 Poinsett Highway Greenville, SC 29609 — 1100 (Single Family). Record owner 2501 Poinsette Llc. Last transfer 05/02/2022 for $130,000. County FMV $306,870.00. Judgment $301,030.64. Debt is 98% of FMV — thin margin. DEFICIENCY DEMANDED — open 30 days.</t>
         </is>
       </c>
     </row>
@@ -4159,7 +4261,9 @@
           <t>waived</t>
         </is>
       </c>
-      <c r="K36" s="12" t="n"/>
+      <c r="K36" s="12" t="n">
+        <v>221056.42</v>
+      </c>
       <c r="L36" s="10" t="n"/>
       <c r="M36" s="12" t="n"/>
       <c r="N36" s="11">
@@ -4200,7 +4304,11 @@
           <t>05/16/2023 $249,900</t>
         </is>
       </c>
-      <c r="Y36" s="11" t="n"/>
+      <c r="Y36" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z36" s="14" t="inlineStr">
         <is>
           <t>open</t>
@@ -4214,7 +4322,7 @@
       </c>
       <c r="AC36" s="9" t="inlineStr">
         <is>
-          <t>202 Port Road Greenville, SC 29617 — 1100 (Single Family) — 0.590 ac (River Valley). Record owner Green Ant Llc. Last transfer 05/16/2023 for $249,900. County FMV $249,890.00. Judgment $ not pulled yet (needs the PC run). Deficiency waived — final on the day.</t>
+          <t>202 Port Road Greenville, SC 29617 — 1100 (Single Family) — 0.590 ac (River Valley). Record owner Green Ant Llc. Last transfer 05/16/2023 for $249,900. County FMV $249,890.00. Judgment $221,056.42. Debt is 88% of FMV — thin margin. Deficiency waived — final on the day.</t>
         </is>
       </c>
     </row>
@@ -11128,131 +11236,149 @@
   <autoFilter ref="A1:AC123"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z9" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y38" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y39" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y42" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y43" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y44" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y45" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y46" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y47" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y48" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y49" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y52" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y54" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y55" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y57" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y58" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y60" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y61" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y62" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y63" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y64" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y65" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y66" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y67" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y68" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y69" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y70" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y71" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y72" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y73" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y10" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y16" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y17" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y18" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB18" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y19" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y20" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y24" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB24" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y26" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB26" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y28" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y31" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB31" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y32" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y33" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB33" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y34" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB34" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y35" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y36" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y38" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y39" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y40" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y41" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y42" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y43" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y44" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y45" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y46" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y47" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y48" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y49" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y50" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y51" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y52" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y53" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y54" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y55" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y56" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y57" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y58" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y59" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y60" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y61" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y62" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y63" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y64" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y65" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y66" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y67" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y68" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y69" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y70" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y71" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y72" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y73" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId144"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
foreclosures: extractor fixes from a real Pickens order + Pickens 9/8 Form 4 amounts
The 103 Windamere Ct order (2024-CP-39-00316) exposed three extractor bugs:
the total picked the principal line ('amount due and owing … Principal $'),
'Per Diem: $ 6.50' was missed, and a 40-char window cut '$ 40,408.88' to
'$ 40'. Total patterns are now tried most-specific-first, the window always
finishes the number it started, 'as of today's date:' and mm/dd/yyyy dates
are accepted, and 'Principal due' beats the note's original principal.
Verified: total 66,266.33 · as of Jul 9 2026 · per diem 6.50 · fees 4,800 ·
waived. Pickens #2/#3/#4 judgment totals (Brian) saved to a seed.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017rdAjmKGDVGAtDqQodYkcB
</commit_message>
<xml_diff>
--- a/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
+++ b/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
@@ -7482,12 +7482,18 @@
       </c>
       <c r="J78" s="11" t="inlineStr">
         <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="K78" s="12" t="n"/>
-      <c r="L78" s="10" t="n"/>
-      <c r="M78" s="12" t="n"/>
+          <t>waived</t>
+        </is>
+      </c>
+      <c r="K78" s="12" t="n">
+        <v>66266.33</v>
+      </c>
+      <c r="L78" s="10" t="n">
+        <v>46212</v>
+      </c>
+      <c r="M78" s="12" t="n">
+        <v>6.5</v>
+      </c>
       <c r="N78" s="11">
         <f>IF(OR(B78="",L78=""),"",MAX(0,B78-L78))</f>
         <v/>
@@ -7496,7 +7502,11 @@
         <f>IF(K78="","",K78+IF(OR(M78="",N78=""),0,M78*N78))</f>
         <v/>
       </c>
-      <c r="P78" s="11" t="n"/>
+      <c r="P78" s="11" t="inlineStr">
+        <is>
+          <t>5.875%</t>
+        </is>
+      </c>
       <c r="Q78" s="12" t="n"/>
       <c r="R78" s="13">
         <f>IF(OR(Q78="",Q78=0,O78=""),"",O78/Q78)</f>
@@ -7508,13 +7518,17 @@
       <c r="V78" s="11" t="n"/>
       <c r="W78" s="11" t="n"/>
       <c r="X78" s="11" t="inlineStr"/>
-      <c r="Y78" s="11" t="n"/>
+      <c r="Y78" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z78" s="11" t="n"/>
       <c r="AA78" s="11" t="n"/>
       <c r="AB78" s="11" t="n"/>
       <c r="AC78" s="9" t="inlineStr">
         <is>
-          <t>103 WINDAMERE CT., EASLEY, SC 29640. Judgment $ not pulled yet (needs the PC run). Deficiency not stated — check the notice.</t>
+          <t>103 WINDAMERE CT., EASLEY, SC 29640. Judgment $66,266.33 as of July 9, 2026 + $6.50/day ≈ $66,662.83 on sale day (5.875%). Deficiency waived — final on the day. Interest on bid 5.875% until compliance; 5% deposit day of sale. Lot 53, Burdine Springs Sec. 2 (City of Easley). Estate case: both borrowers deceased, PR Heather Howell in default. First lien; sold subject to taxes/assessments only. Interest on bid 5.875% to compliance.</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7579,9 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K79" s="12" t="n"/>
+      <c r="K79" s="12" t="n">
+        <v>223932.51</v>
+      </c>
       <c r="L79" s="10" t="n"/>
       <c r="M79" s="12" t="n"/>
       <c r="N79" s="11">
@@ -7588,13 +7604,17 @@
       <c r="V79" s="11" t="n"/>
       <c r="W79" s="11" t="n"/>
       <c r="X79" s="11" t="inlineStr"/>
-      <c r="Y79" s="11" t="n"/>
+      <c r="Y79" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z79" s="11" t="n"/>
       <c r="AA79" s="11" t="n"/>
       <c r="AB79" s="11" t="n"/>
       <c r="AC79" s="9" t="inlineStr">
         <is>
-          <t>649 N. NORRIS DR., LIBERTY, SC 29657. Judgment $ not pulled yet (needs the PC run). Deficiency not stated — check the notice.</t>
+          <t>649 N. NORRIS DR., LIBERTY, SC 29657. Judgment $223,932.51. Deficiency not stated — check the notice.</t>
         </is>
       </c>
     </row>
@@ -7645,7 +7665,9 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K80" s="12" t="n"/>
+      <c r="K80" s="12" t="n">
+        <v>623367.66</v>
+      </c>
       <c r="L80" s="10" t="n"/>
       <c r="M80" s="12" t="n"/>
       <c r="N80" s="11">
@@ -7668,13 +7690,17 @@
       <c r="V80" s="11" t="n"/>
       <c r="W80" s="11" t="n"/>
       <c r="X80" s="11" t="inlineStr"/>
-      <c r="Y80" s="11" t="n"/>
+      <c r="Y80" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z80" s="11" t="n"/>
       <c r="AA80" s="11" t="n"/>
       <c r="AB80" s="11" t="n"/>
       <c r="AC80" s="9" t="inlineStr">
         <is>
-          <t>365 GIBSON RD., EASLEY, SC 29640. Judgment $ not pulled yet (needs the PC run). Deficiency not stated — check the notice.</t>
+          <t>365 GIBSON RD., EASLEY, SC 29640. Judgment $623,367.66. Deficiency not stated — check the notice.</t>
         </is>
       </c>
     </row>
@@ -11339,46 +11365,49 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y78" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y79" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y80" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId147"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Foreclosures: extractor fixes from a real Pickens order + Pickens 9/8 Form 4 amounts (#76)
The 103 Windamere Ct order (2024-CP-39-00316) exposed three extractor bugs:
the total picked the principal line ('amount due and owing … Principal $'),
'Per Diem: $ 6.50' was missed, and a 40-char window cut '$ 40,408.88' to
'$ 40'. Total patterns are now tried most-specific-first, the window always
finishes the number it started, 'as of today's date:' and mm/dd/yyyy dates
are accepted, and 'Principal due' beats the note's original principal.
Verified: total 66,266.33 · as of Jul 9 2026 · per diem 6.50 · fees 4,800 ·
waived. Pickens #2/#3/#4 judgment totals (Brian) saved to a seed.


Claude-Session: https://claude.ai/code/session_017rdAjmKGDVGAtDqQodYkcB

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
+++ b/tools/foreclosures/reports/SC-foreclosures-2026-09.xlsx
@@ -7482,12 +7482,18 @@
       </c>
       <c r="J78" s="11" t="inlineStr">
         <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="K78" s="12" t="n"/>
-      <c r="L78" s="10" t="n"/>
-      <c r="M78" s="12" t="n"/>
+          <t>waived</t>
+        </is>
+      </c>
+      <c r="K78" s="12" t="n">
+        <v>66266.33</v>
+      </c>
+      <c r="L78" s="10" t="n">
+        <v>46212</v>
+      </c>
+      <c r="M78" s="12" t="n">
+        <v>6.5</v>
+      </c>
       <c r="N78" s="11">
         <f>IF(OR(B78="",L78=""),"",MAX(0,B78-L78))</f>
         <v/>
@@ -7496,7 +7502,11 @@
         <f>IF(K78="","",K78+IF(OR(M78="",N78=""),0,M78*N78))</f>
         <v/>
       </c>
-      <c r="P78" s="11" t="n"/>
+      <c r="P78" s="11" t="inlineStr">
+        <is>
+          <t>5.875%</t>
+        </is>
+      </c>
       <c r="Q78" s="12" t="n"/>
       <c r="R78" s="13">
         <f>IF(OR(Q78="",Q78=0,O78=""),"",O78/Q78)</f>
@@ -7508,13 +7518,17 @@
       <c r="V78" s="11" t="n"/>
       <c r="W78" s="11" t="n"/>
       <c r="X78" s="11" t="inlineStr"/>
-      <c r="Y78" s="11" t="n"/>
+      <c r="Y78" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z78" s="11" t="n"/>
       <c r="AA78" s="11" t="n"/>
       <c r="AB78" s="11" t="n"/>
       <c r="AC78" s="9" t="inlineStr">
         <is>
-          <t>103 WINDAMERE CT., EASLEY, SC 29640. Judgment $ not pulled yet (needs the PC run). Deficiency not stated — check the notice.</t>
+          <t>103 WINDAMERE CT., EASLEY, SC 29640. Judgment $66,266.33 as of July 9, 2026 + $6.50/day ≈ $66,662.83 on sale day (5.875%). Deficiency waived — final on the day. Interest on bid 5.875% until compliance; 5% deposit day of sale. Lot 53, Burdine Springs Sec. 2 (City of Easley). Estate case: both borrowers deceased, PR Heather Howell in default. First lien; sold subject to taxes/assessments only. Interest on bid 5.875% to compliance.</t>
         </is>
       </c>
     </row>
@@ -7565,7 +7579,9 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K79" s="12" t="n"/>
+      <c r="K79" s="12" t="n">
+        <v>223932.51</v>
+      </c>
       <c r="L79" s="10" t="n"/>
       <c r="M79" s="12" t="n"/>
       <c r="N79" s="11">
@@ -7588,13 +7604,17 @@
       <c r="V79" s="11" t="n"/>
       <c r="W79" s="11" t="n"/>
       <c r="X79" s="11" t="inlineStr"/>
-      <c r="Y79" s="11" t="n"/>
+      <c r="Y79" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z79" s="11" t="n"/>
       <c r="AA79" s="11" t="n"/>
       <c r="AB79" s="11" t="n"/>
       <c r="AC79" s="9" t="inlineStr">
         <is>
-          <t>649 N. NORRIS DR., LIBERTY, SC 29657. Judgment $ not pulled yet (needs the PC run). Deficiency not stated — check the notice.</t>
+          <t>649 N. NORRIS DR., LIBERTY, SC 29657. Judgment $223,932.51. Deficiency not stated — check the notice.</t>
         </is>
       </c>
     </row>
@@ -7645,7 +7665,9 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="K80" s="12" t="n"/>
+      <c r="K80" s="12" t="n">
+        <v>623367.66</v>
+      </c>
       <c r="L80" s="10" t="n"/>
       <c r="M80" s="12" t="n"/>
       <c r="N80" s="11">
@@ -7668,13 +7690,17 @@
       <c r="V80" s="11" t="n"/>
       <c r="W80" s="11" t="n"/>
       <c r="X80" s="11" t="inlineStr"/>
-      <c r="Y80" s="11" t="n"/>
+      <c r="Y80" s="14" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
       <c r="Z80" s="11" t="n"/>
       <c r="AA80" s="11" t="n"/>
       <c r="AB80" s="11" t="n"/>
       <c r="AC80" s="9" t="inlineStr">
         <is>
-          <t>365 GIBSON RD., EASLEY, SC 29640. Judgment $ not pulled yet (needs the PC run). Deficiency not stated — check the notice.</t>
+          <t>365 GIBSON RD., EASLEY, SC 29640. Judgment $623,367.66. Deficiency not stated — check the notice.</t>
         </is>
       </c>
     </row>
@@ -11339,46 +11365,49 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y74" r:id="rId102"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y75" r:id="rId103"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y76" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y78" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y79" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y80" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y115" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y116" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y117" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y118" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y119" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y120" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y121" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y122" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Y123" r:id="rId147"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>